<commit_message>
tinghare baato estimate corrected
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर estimate/तिनघरे बाटो स्तरोन्नति/तिनघरे बाटो स्तरोन्नति.xlsx
+++ b/बजेट माग estimate/नगर estimate/तिनघरे बाटो स्तरोन्नति/तिनघरे बाटो स्तरोन्नति.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ABED650-AEA0-42DD-B8F2-EDA139EAAB54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89090C2C-84C9-4C4D-A73A-172EBC4DC784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$46</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'small wall'!$A$1:$K$49</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'small wall'!$1:$8</definedName>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="44">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -187,6 +187,15 @@
   </si>
   <si>
     <t>-13% VAT for stone</t>
+  </si>
+  <si>
+    <t>Earthwork Excavation in Cutting., Roadway Excavation in all types of Soil by Mechanical  Means ., Road way Excavation in  all types of soil as per Drawing and technical specifications  including  removal of stumps and other deleterious matter and backfilling, all lifts and lead as per Drawing and instruction of the Engineer.</t>
+  </si>
+  <si>
+    <t>-13% VAT for water</t>
+  </si>
+  <si>
+    <t>User contribution</t>
   </si>
 </sst>
 </file>
@@ -356,7 +365,7 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -446,24 +455,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -483,7 +474,24 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1013,7 +1021,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:S45"/>
+  <dimension ref="A1:S46"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
@@ -1025,120 +1033,120 @@
     <col min="7" max="7" width="9.140625" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.5703125" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="9.140625" style="19"/>
     <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
     <col min="17" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
     </row>
     <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
     </row>
     <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="37"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="38" t="s">
+      <c r="H6" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
+      <c r="I6" s="45"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="45"/>
     </row>
     <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="46" t="s">
+      <c r="H7" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="46"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="40"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -1175,13 +1183,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="189" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="188.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
         <v>1</v>
       </c>
-      <c r="B9" s="35" t="str">
-        <f>description_276</f>
-        <v>Excavation for Structures Foundation, Earth work in excavation of foundation of structures, including  construction of shoring and bracing, removal of stumps and other deleterious matter and backfilling with approved Material as per Drawing and Technical Specifications., Ordinary soil by Mechanical Means, Depth upto 3 m</v>
+      <c r="B9" s="35" t="s">
+        <v>41</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
@@ -1250,11 +1257,11 @@
         <v>18</v>
       </c>
       <c r="I11" s="6">
-        <v>94.43</v>
+        <v>62.95</v>
       </c>
       <c r="J11" s="18">
         <f>G11*I11</f>
-        <v>7861.2975000000006</v>
+        <v>5240.5875000000005</v>
       </c>
       <c r="K11" s="5"/>
     </row>
@@ -1271,8 +1278,8 @@
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
       <c r="J12" s="18">
-        <f>0.13*G11*(18612)/240</f>
-        <v>839.28487499999994</v>
+        <f>0.13*G11*(18612)/360</f>
+        <v>559.52324999999996</v>
       </c>
       <c r="K12" s="17"/>
     </row>
@@ -1289,7 +1296,7 @@
       <c r="J13" s="17"/>
       <c r="K13" s="17"/>
     </row>
-    <row r="14" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A14" s="16">
         <v>2</v>
       </c>
@@ -1404,7 +1411,7 @@
       <c r="J18" s="17"/>
       <c r="K18" s="17"/>
     </row>
-    <row r="19" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A19" s="16">
         <v>3</v>
       </c>
@@ -1591,7 +1598,9 @@
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
-      <c r="B27" s="17"/>
+      <c r="B27" s="32" t="s">
+        <v>42</v>
+      </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="17"/>
@@ -1599,16 +1608,15 @@
       <c r="G27" s="17"/>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
+      <c r="J27" s="18">
+        <f>0.13*G22*(310)/5</f>
+        <v>14.538225000000002</v>
+      </c>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="A28" s="16">
-        <v>4</v>
-      </c>
-      <c r="B28" s="35" t="s">
-        <v>39</v>
-      </c>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="16"/>
+      <c r="B28" s="17"/>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
       <c r="E28" s="17"/>
@@ -1619,76 +1627,64 @@
       <c r="J28" s="17"/>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="16"/>
-      <c r="B29" s="32" t="str">
-        <f>B20</f>
-        <v>-for masonary wall</v>
-      </c>
-      <c r="C29" s="17">
-        <v>1</v>
-      </c>
-      <c r="D29" s="33">
-        <f>D10</f>
-        <v>18.5</v>
-      </c>
-      <c r="E29" s="33">
-        <f>((F29/2)+0.45)/2</f>
-        <v>0.97499999999999998</v>
-      </c>
-      <c r="F29" s="33">
-        <v>3</v>
-      </c>
-      <c r="G29" s="33">
-        <f>PRODUCT(C29:F29)</f>
-        <v>54.112499999999997</v>
-      </c>
+    <row r="29" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A29" s="16">
+        <v>4</v>
+      </c>
+      <c r="B29" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
       <c r="H29" s="17"/>
       <c r="I29" s="17"/>
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
-      <c r="M29" s="33">
-        <f>7</f>
-        <v>7</v>
-      </c>
-      <c r="N29" s="33">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="O29" s="33"/>
-      <c r="P29" s="33">
-        <f>PI()*M29*SQRT(M29^2+N29^2)</f>
-        <v>160.09797821843054</v>
-      </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
-      <c r="B30" s="32"/>
+      <c r="B30" s="32" t="str">
+        <f>B20</f>
+        <v>-for masonary wall</v>
+      </c>
       <c r="C30" s="17">
         <v>1</v>
       </c>
       <c r="D30" s="33">
-        <f>D29</f>
+        <f>D10</f>
         <v>18.5</v>
       </c>
       <c r="E30" s="33">
-        <v>0.45</v>
+        <f>((F30/2)+0.45)/2</f>
+        <v>0.97499999999999998</v>
       </c>
       <c r="F30" s="33">
-        <v>0.05</v>
+        <v>3</v>
       </c>
       <c r="G30" s="33">
         <f>PRODUCT(C30:F30)</f>
-        <v>0.41625000000000006</v>
+        <v>54.112499999999997</v>
       </c>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
       <c r="J30" s="17"/>
       <c r="K30" s="17"/>
-      <c r="M30" s="36"/>
-      <c r="N30" s="36"/>
-      <c r="O30" s="36"/>
-      <c r="P30" s="36"/>
+      <c r="M30" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N30" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O30" s="33"/>
+      <c r="P30" s="33">
+        <f>PI()*M30*SQRT(M30^2+N30^2)</f>
+        <v>160.09797821843054</v>
+      </c>
     </row>
     <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
@@ -1700,8 +1696,8 @@
       <c r="E31" s="5"/>
       <c r="F31" s="5"/>
       <c r="G31" s="6">
-        <f>SUM(G29:G30)</f>
-        <v>54.528749999999995</v>
+        <f>SUM(G30:G30)</f>
+        <v>54.112499999999997</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>18</v>
@@ -1711,7 +1707,7 @@
       </c>
       <c r="J31" s="18">
         <f>G31*I31</f>
-        <v>490095.13511249993</v>
+        <v>486353.95087499998</v>
       </c>
       <c r="K31" s="5"/>
     </row>
@@ -1729,7 +1725,7 @@
       <c r="I32" s="17"/>
       <c r="J32" s="18">
         <f>0.13*G31*(5863.95)/5</f>
-        <v>8313.6004526249999</v>
+        <v>8250.1378537500004</v>
       </c>
       <c r="K32" s="17"/>
     </row>
@@ -1747,7 +1743,7 @@
       <c r="I33" s="17"/>
       <c r="J33" s="18">
         <f>0.13*G31*(6604.416)/5</f>
-        <v>9363.3942729599985</v>
+        <v>9291.9179808000008</v>
       </c>
       <c r="K33" s="17"/>
     </row>
@@ -1765,13 +1761,15 @@
       <c r="I34" s="17"/>
       <c r="J34" s="18">
         <f>0.13*G31*(14808.78)/5</f>
-        <v>20995.110823049999</v>
+        <v>20834.842801500003</v>
       </c>
       <c r="K34" s="17"/>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
-      <c r="B35" s="17"/>
+      <c r="B35" s="32" t="s">
+        <v>42</v>
+      </c>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
       <c r="E35" s="17"/>
@@ -1779,179 +1777,187 @@
       <c r="G35" s="17"/>
       <c r="H35" s="17"/>
       <c r="I35" s="17"/>
-      <c r="J35" s="17"/>
+      <c r="J35" s="18">
+        <f>0.13*G31*(310)/5</f>
+        <v>436.14675</v>
+      </c>
       <c r="K35" s="17"/>
     </row>
-    <row r="36" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A36" s="16"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="17"/>
+    </row>
+    <row r="37" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
         <v>5</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B37" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C36" s="3">
+      <c r="C37" s="3">
         <v>1</v>
       </c>
-      <c r="D36" s="4"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="7">
-        <f t="shared" ref="G36" si="0">PRODUCT(C36:F36)</f>
-        <v>1</v>
-      </c>
-      <c r="H36" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I36" s="6">
-        <v>500</v>
-      </c>
-      <c r="J36" s="7">
-        <f>G36*I36</f>
-        <v>500</v>
-      </c>
-      <c r="K36" s="5"/>
-    </row>
-    <row r="37" spans="1:19" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="2"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="3"/>
       <c r="D37" s="4"/>
       <c r="E37" s="5"/>
       <c r="F37" s="5"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="18"/>
+      <c r="G37" s="7">
+        <f t="shared" ref="G37" si="0">PRODUCT(C37:F37)</f>
+        <v>1</v>
+      </c>
+      <c r="H37" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I37" s="6">
+        <v>500</v>
+      </c>
+      <c r="J37" s="7">
+        <f>G37*I37</f>
+        <v>500</v>
+      </c>
       <c r="K37" s="5"/>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A38" s="21"/>
-      <c r="B38" s="22" t="s">
+      <c r="A38" s="2"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="6"/>
+      <c r="J38" s="18"/>
+      <c r="K38" s="5"/>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A39" s="21"/>
+      <c r="B39" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="C38" s="23"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="24"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
-      <c r="I38" s="18"/>
-      <c r="J38" s="18">
-        <f>SUM(J9:J36)</f>
-        <v>579863.69240950991</v>
-      </c>
-      <c r="K38" s="25"/>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M39" s="20"/>
-      <c r="N39" s="20"/>
-      <c r="O39" s="20"/>
-      <c r="P39" s="20"/>
-      <c r="Q39" s="20"/>
-      <c r="R39" s="20"/>
-      <c r="S39" s="20"/>
-    </row>
-    <row r="40" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="26"/>
-      <c r="B40" s="27" t="s">
+      <c r="C39" s="23"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
+      <c r="J39" s="18">
+        <f>SUM(J9:J37)</f>
+        <v>573377.51460942498</v>
+      </c>
+      <c r="K39" s="25"/>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="M40" s="20"/>
+      <c r="N40" s="20"/>
+      <c r="O40" s="20"/>
+      <c r="P40" s="20"/>
+      <c r="Q40" s="20"/>
+      <c r="R40" s="20"/>
+      <c r="S40" s="20"/>
+    </row>
+    <row r="41" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="26"/>
+      <c r="B41" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C40" s="43">
-        <f>J38</f>
-        <v>579863.69240950991</v>
-      </c>
-      <c r="D40" s="44"/>
-      <c r="E40" s="9">
+      <c r="C41" s="37">
+        <f>J39</f>
+        <v>573377.51460942498</v>
+      </c>
+      <c r="D41" s="38"/>
+      <c r="E41" s="9">
         <v>100</v>
       </c>
-      <c r="F40" s="26"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="26"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="30"/>
-      <c r="K40" s="31"/>
-      <c r="M40" s="19"/>
-      <c r="N40" s="19"/>
-      <c r="O40" s="19"/>
-      <c r="P40" s="19"/>
-      <c r="Q40" s="19"/>
-      <c r="R40" s="19"/>
-      <c r="S40" s="19"/>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B41" s="27" t="s">
-        <v>25</v>
-      </c>
-      <c r="C41" s="47">
-        <v>500000</v>
-      </c>
-      <c r="D41" s="48"/>
-      <c r="E41" s="9"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="26"/>
+      <c r="I41" s="29"/>
+      <c r="J41" s="30"/>
+      <c r="K41" s="31"/>
+      <c r="M41" s="19"/>
+      <c r="N41" s="19"/>
+      <c r="O41" s="19"/>
+      <c r="P41" s="19"/>
+      <c r="Q41" s="19"/>
+      <c r="R41" s="19"/>
+      <c r="S41" s="19"/>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B42" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="C42" s="47">
-        <f>C41-C44-C45</f>
-        <v>475000</v>
-      </c>
-      <c r="D42" s="48"/>
-      <c r="E42" s="9">
-        <f>C42/C40*100</f>
-        <v>81.915803009881614</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="C42" s="41">
+        <v>500000</v>
+      </c>
+      <c r="D42" s="42"/>
+      <c r="E42" s="9"/>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B43" s="27" t="s">
-        <v>30</v>
-      </c>
-      <c r="C43" s="49">
-        <f>C40-C42</f>
-        <v>104863.69240950991</v>
-      </c>
-      <c r="D43" s="49"/>
+        <v>26</v>
+      </c>
+      <c r="C43" s="41">
+        <f>C42-C45-C46</f>
+        <v>475000</v>
+      </c>
+      <c r="D43" s="42"/>
       <c r="E43" s="9">
-        <f>100-E42</f>
-        <v>18.084196990118386</v>
+        <f>C43/C41*100</f>
+        <v>82.842453339587607</v>
       </c>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B44" s="27" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="C44" s="43">
-        <f>C41*0.03</f>
-        <v>15000</v>
-      </c>
-      <c r="D44" s="44"/>
+        <f>C41-C43</f>
+        <v>98377.514609424979</v>
+      </c>
+      <c r="D44" s="43"/>
       <c r="E44" s="9">
-        <v>3</v>
+        <f>100-E43</f>
+        <v>17.157546660412393</v>
       </c>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B45" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C45" s="37">
+        <f>C42*0.03</f>
+        <v>15000</v>
+      </c>
+      <c r="D45" s="38"/>
+      <c r="E45" s="9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B46" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C45" s="43">
-        <f>C41*0.02</f>
+      <c r="C46" s="37">
+        <f>C42*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D45" s="44"/>
-      <c r="E45" s="9">
+      <c r="D46" s="38"/>
+      <c r="E46" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C44:D44"/>
-    <mergeCell ref="C45:D45"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C41:D41"/>
-    <mergeCell ref="C42:D42"/>
-    <mergeCell ref="C43:D43"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -1959,12 +1965,23 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C44:D44"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="28" max="10" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
 
@@ -1989,113 +2006,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
     </row>
     <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
     </row>
     <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="37"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="38" t="s">
+      <c r="H6" s="45" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
+      <c r="I6" s="45"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="45"/>
     </row>
     <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="46" t="s">
+      <c r="H7" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="46"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="40"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -2215,10 +2232,10 @@
       <c r="I11" s="17"/>
       <c r="J11" s="17"/>
       <c r="K11" s="17"/>
-      <c r="M11" s="50"/>
-      <c r="N11" s="50"/>
-      <c r="O11" s="50"/>
-      <c r="P11" s="50"/>
+      <c r="M11" s="36"/>
+      <c r="N11" s="36"/>
+      <c r="O11" s="36"/>
+      <c r="P11" s="36"/>
     </row>
     <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
@@ -2360,10 +2377,10 @@
       <c r="I17" s="17"/>
       <c r="J17" s="17"/>
       <c r="K17" s="17"/>
-      <c r="M17" s="50"/>
-      <c r="N17" s="50"/>
-      <c r="O17" s="50"/>
-      <c r="P17" s="50"/>
+      <c r="M17" s="36"/>
+      <c r="N17" s="36"/>
+      <c r="O17" s="36"/>
+      <c r="P17" s="36"/>
     </row>
     <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
@@ -2773,10 +2790,10 @@
       <c r="I34" s="17"/>
       <c r="J34" s="17"/>
       <c r="K34" s="17"/>
-      <c r="M34" s="50"/>
-      <c r="N34" s="50"/>
-      <c r="O34" s="50"/>
-      <c r="P34" s="50"/>
+      <c r="M34" s="36"/>
+      <c r="N34" s="36"/>
+      <c r="O34" s="36"/>
+      <c r="P34" s="36"/>
     </row>
     <row r="35" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
@@ -2944,11 +2961,11 @@
       <c r="B44" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C44" s="43">
+      <c r="C44" s="37">
         <f>J42</f>
         <v>570250.82872341503</v>
       </c>
-      <c r="D44" s="44"/>
+      <c r="D44" s="38"/>
       <c r="E44" s="9">
         <v>100</v>
       </c>
@@ -2970,21 +2987,21 @@
       <c r="B45" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C45" s="47">
+      <c r="C45" s="41">
         <v>500000</v>
       </c>
-      <c r="D45" s="48"/>
+      <c r="D45" s="42"/>
       <c r="E45" s="9"/>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B46" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C46" s="47">
+      <c r="C46" s="41">
         <f>C45-C48-C49</f>
         <v>475000</v>
       </c>
-      <c r="D46" s="48"/>
+      <c r="D46" s="42"/>
       <c r="E46" s="9">
         <f>C46/C44*100</f>
         <v>83.296678597267956</v>
@@ -2994,11 +3011,11 @@
       <c r="B47" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="C47" s="49">
+      <c r="C47" s="43">
         <f>C44-C46</f>
         <v>95250.828723415034</v>
       </c>
-      <c r="D47" s="49"/>
+      <c r="D47" s="43"/>
       <c r="E47" s="9">
         <f>100-E46</f>
         <v>16.703321402732044</v>
@@ -3008,11 +3025,11 @@
       <c r="B48" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C48" s="43">
+      <c r="C48" s="37">
         <f>C45*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D48" s="44"/>
+      <c r="D48" s="38"/>
       <c r="E48" s="9">
         <v>3</v>
       </c>
@@ -3021,17 +3038,24 @@
       <c r="B49" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C49" s="43">
+      <c r="C49" s="37">
         <f>C45*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D49" s="44"/>
+      <c r="D49" s="38"/>
       <c r="E49" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="C49:D49"/>
     <mergeCell ref="A7:F7"/>
@@ -3040,13 +3064,6 @@
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="C47:D47"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>

</xml_diff>